<commit_message>
Rationale per answer, policy viewer with highlighted quote and version diff, logo loading mark, CAIQ domain context, pitch pack
</commit_message>
<xml_diff>
--- a/benchmark/answer_key_filled.xlsx
+++ b/benchmark/answer_key_filled.xlsx
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="M7" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N7" s="4" t="n"/>
       <c r="O7" s="4" t="n"/>
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n"/>
       <c r="O10" s="4" t="n"/>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="M13" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N13" s="4" t="n"/>
       <c r="O13" s="4" t="n"/>
@@ -2293,7 +2293,7 @@
         </is>
       </c>
       <c r="M30" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N30" s="4" t="n"/>
       <c r="O30" s="4" t="n"/>
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="M40" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N40" s="4" t="n"/>
       <c r="O40" s="4" t="n"/>
@@ -3421,7 +3421,7 @@
         </is>
       </c>
       <c r="M48" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N48" s="4" t="n"/>
       <c r="O48" s="4" t="n"/>
@@ -3686,7 +3686,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>20.3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="58">
@@ -3696,7 +3696,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.021</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="59">

</xml_diff>

<commit_message>
Final benchmark, pitch pack and submission from measured numbers, viewer scroll
</commit_message>
<xml_diff>
--- a/benchmark/answer_key_filled.xlsx
+++ b/benchmark/answer_key_filled.xlsx
@@ -636,16 +636,16 @@
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
         </is>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="4" t="n"/>
       <c r="O4" s="4" t="n"/>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N7" s="4" t="n"/>
       <c r="O7" s="4" t="n"/>
@@ -961,11 +961,11 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>green</t>
         </is>
       </c>
       <c r="M9" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N9" s="4" t="n"/>
       <c r="O9" s="4" t="n"/>
@@ -1021,11 +1021,11 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N10" s="4" t="n"/>
       <c r="O10" s="4" t="n"/>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N13" s="4" t="n"/>
       <c r="O13" s="4" t="n"/>
@@ -2028,16 +2028,16 @@
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>red</t>
         </is>
       </c>
       <c r="M26" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N26" s="4" t="n"/>
       <c r="O26" s="4" t="n"/>
@@ -2293,7 +2293,7 @@
         </is>
       </c>
       <c r="M30" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N30" s="4" t="n"/>
       <c r="O30" s="4" t="n"/>
@@ -3045,11 +3045,11 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="M42" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N42" s="4" t="n"/>
       <c r="O42" s="4" t="n"/>
@@ -3686,7 +3686,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>16</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
Measured closed-model baseline (OpenAI gpt-6-sol) in benchmark, docs, deck
</commit_message>
<xml_diff>
--- a/benchmark/answer_key_filled.xlsx
+++ b/benchmark/answer_key_filled.xlsx
@@ -523,9 +523,19 @@
       <c r="M2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N2" s="4" t="n"/>
-      <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -587,9 +597,19 @@
       <c r="M3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N3" s="4" t="n"/>
-      <c r="O3" s="4" t="n"/>
-      <c r="P3" s="4" t="n"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -647,9 +667,19 @@
       <c r="M4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="n"/>
-      <c r="P4" s="4" t="n"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -711,9 +741,19 @@
       <c r="M5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N5" s="4" t="n"/>
-      <c r="O5" s="4" t="n"/>
-      <c r="P5" s="4" t="n"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -771,9 +811,19 @@
       <c r="M6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N6" s="4" t="n"/>
-      <c r="O6" s="4" t="n"/>
-      <c r="P6" s="4" t="n"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -835,9 +885,19 @@
       <c r="M7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="4" t="n"/>
-      <c r="O7" s="4" t="n"/>
-      <c r="P7" s="4" t="n"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -899,9 +959,19 @@
       <c r="M8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N8" s="4" t="n"/>
-      <c r="O8" s="4" t="n"/>
-      <c r="P8" s="4" t="n"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -967,9 +1037,19 @@
       <c r="M9" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="N9" s="4" t="n"/>
-      <c r="O9" s="4" t="n"/>
-      <c r="P9" s="4" t="n"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1027,9 +1107,19 @@
       <c r="M10" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="N10" s="4" t="n"/>
-      <c r="O10" s="4" t="n"/>
-      <c r="P10" s="4" t="n"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1093,11 +1183,21 @@
         </is>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N11" s="4" t="n"/>
-      <c r="O11" s="4" t="n"/>
-      <c r="P11" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1157,15 +1257,25 @@
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="M12" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N12" s="4" t="n"/>
-      <c r="O12" s="4" t="n"/>
-      <c r="P12" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1227,9 +1337,19 @@
       <c r="M13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N13" s="4" t="n"/>
-      <c r="O13" s="4" t="n"/>
-      <c r="P13" s="4" t="n"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1287,9 +1407,19 @@
       <c r="M14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N14" s="4" t="n"/>
-      <c r="O14" s="4" t="n"/>
-      <c r="P14" s="4" t="n"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1351,9 +1481,19 @@
       <c r="M15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N15" s="4" t="n"/>
-      <c r="O15" s="4" t="n"/>
-      <c r="P15" s="4" t="n"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1415,9 +1555,19 @@
       <c r="M16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N16" s="4" t="n"/>
-      <c r="O16" s="4" t="n"/>
-      <c r="P16" s="4" t="n"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1483,9 +1633,19 @@
       <c r="M17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N17" s="4" t="n"/>
-      <c r="O17" s="4" t="n"/>
-      <c r="P17" s="4" t="n"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1543,9 +1703,19 @@
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N18" s="4" t="n"/>
-      <c r="O18" s="4" t="n"/>
-      <c r="P18" s="4" t="n"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1607,9 +1777,19 @@
       <c r="M19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="4" t="n"/>
-      <c r="O19" s="4" t="n"/>
-      <c r="P19" s="4" t="n"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1667,9 +1847,19 @@
       <c r="M20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N20" s="4" t="n"/>
-      <c r="O20" s="4" t="n"/>
-      <c r="P20" s="4" t="n"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1731,9 +1921,19 @@
       <c r="M21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N21" s="4" t="n"/>
-      <c r="O21" s="4" t="n"/>
-      <c r="P21" s="4" t="n"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1791,9 +1991,19 @@
       <c r="M22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N22" s="4" t="n"/>
-      <c r="O22" s="4" t="n"/>
-      <c r="P22" s="4" t="n"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1855,9 +2065,19 @@
       <c r="M23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N23" s="4" t="n"/>
-      <c r="O23" s="4" t="n"/>
-      <c r="P23" s="4" t="n"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1919,9 +2139,19 @@
       <c r="M24" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N24" s="4" t="n"/>
-      <c r="O24" s="4" t="n"/>
-      <c r="P24" s="4" t="n"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1977,11 +2207,21 @@
         </is>
       </c>
       <c r="M25" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N25" s="4" t="n"/>
-      <c r="O25" s="4" t="n"/>
-      <c r="P25" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2039,9 +2279,19 @@
       <c r="M26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="N26" s="4" t="n"/>
-      <c r="O26" s="4" t="n"/>
-      <c r="P26" s="4" t="n"/>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2103,9 +2353,19 @@
       <c r="M27" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="N27" s="4" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P27" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2167,9 +2427,19 @@
       <c r="M28" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N28" s="4" t="n"/>
-      <c r="O28" s="4" t="n"/>
-      <c r="P28" s="4" t="n"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P28" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2231,9 +2501,19 @@
       <c r="M29" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N29" s="4" t="n"/>
-      <c r="O29" s="4" t="n"/>
-      <c r="P29" s="4" t="n"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P29" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2295,9 +2575,19 @@
       <c r="M30" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N30" s="4" t="n"/>
-      <c r="O30" s="4" t="n"/>
-      <c r="P30" s="4" t="n"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2359,9 +2649,19 @@
       <c r="M31" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N31" s="4" t="n"/>
-      <c r="O31" s="4" t="n"/>
-      <c r="P31" s="4" t="n"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2423,9 +2723,19 @@
       <c r="M32" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N32" s="4" t="n"/>
-      <c r="O32" s="4" t="n"/>
-      <c r="P32" s="4" t="n"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2483,9 +2793,19 @@
       <c r="M33" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N33" s="4" t="n"/>
-      <c r="O33" s="4" t="n"/>
-      <c r="P33" s="4" t="n"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2547,9 +2867,19 @@
       <c r="M34" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="4" t="n"/>
-      <c r="O34" s="4" t="n"/>
-      <c r="P34" s="4" t="n"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P34" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2611,9 +2941,19 @@
       <c r="M35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N35" s="4" t="n"/>
-      <c r="O35" s="4" t="n"/>
-      <c r="P35" s="4" t="n"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2675,9 +3015,19 @@
       <c r="M36" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N36" s="4" t="n"/>
-      <c r="O36" s="4" t="n"/>
-      <c r="P36" s="4" t="n"/>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P36" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2739,9 +3089,19 @@
       <c r="M37" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N37" s="4" t="n"/>
-      <c r="O37" s="4" t="n"/>
-      <c r="P37" s="4" t="n"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2799,9 +3159,19 @@
       <c r="M38" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N38" s="4" t="n"/>
-      <c r="O38" s="4" t="n"/>
-      <c r="P38" s="4" t="n"/>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2863,9 +3233,19 @@
       <c r="M39" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="N39" s="4" t="n"/>
-      <c r="O39" s="4" t="n"/>
-      <c r="P39" s="4" t="n"/>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2927,9 +3307,19 @@
       <c r="M40" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="N40" s="4" t="n"/>
-      <c r="O40" s="4" t="n"/>
-      <c r="P40" s="4" t="n"/>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P40" s="4" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2987,9 +3377,19 @@
       <c r="M41" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N41" s="4" t="n"/>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -3049,11 +3449,21 @@
         </is>
       </c>
       <c r="M42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N42" s="4" t="n"/>
-      <c r="O42" s="4" t="n"/>
-      <c r="P42" s="4" t="n"/>
+        <v>0.5</v>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P42" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -3115,9 +3525,19 @@
       <c r="M43" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N43" s="4" t="n"/>
-      <c r="O43" s="4" t="n"/>
-      <c r="P43" s="4" t="n"/>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P43" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -3175,9 +3595,19 @@
       <c r="M44" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N44" s="4" t="n"/>
-      <c r="O44" s="4" t="n"/>
-      <c r="P44" s="4" t="n"/>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P44" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3239,9 +3669,19 @@
       <c r="M45" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="4" t="n"/>
-      <c r="O45" s="4" t="n"/>
-      <c r="P45" s="4" t="n"/>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P45" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3299,9 +3739,19 @@
       <c r="M46" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N46" s="4" t="n"/>
-      <c r="O46" s="4" t="n"/>
-      <c r="P46" s="4" t="n"/>
+      <c r="N46" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P46" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3363,9 +3813,19 @@
       <c r="M47" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="N47" s="4" t="n"/>
-      <c r="O47" s="4" t="n"/>
-      <c r="P47" s="4" t="n"/>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P47" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3423,9 +3883,19 @@
       <c r="M48" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="4" t="n"/>
-      <c r="O48" s="4" t="n"/>
-      <c r="P48" s="4" t="n"/>
+      <c r="N48" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O48" s="4" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P48" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3487,9 +3957,19 @@
       <c r="M49" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N49" s="4" t="n"/>
-      <c r="O49" s="4" t="n"/>
-      <c r="P49" s="4" t="n"/>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P49" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3551,9 +4031,19 @@
       <c r="M50" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N50" s="4" t="n"/>
-      <c r="O50" s="4" t="n"/>
-      <c r="P50" s="4" t="n"/>
+      <c r="N50" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O50" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P50" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3611,9 +4101,19 @@
       <c r="M51" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N51" s="4" t="n"/>
-      <c r="O51" s="4" t="n"/>
-      <c r="P51" s="4" t="n"/>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P51" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52"/>
     <row r="53">
@@ -3686,7 +4186,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>15.5</v>
+        <v>26.6</v>
+      </c>
+      <c r="E57" t="n">
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="58">
@@ -3697,6 +4200,9 @@
       </c>
       <c r="B58" t="n">
         <v>0.023</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="59">

</xml_diff>